<commit_message>
Remove goal loop from report methodology
</commit_message>
<xml_diff>
--- a/docs/gantt_schedule.xlsx
+++ b/docs/gantt_schedule.xlsx
@@ -763,7 +763,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Goal 기반 설계 루프</t>
+          <t>화면 설계서</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -968,7 +968,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand requirements and implementation methodology
</commit_message>
<xml_diff>
--- a/docs/gantt_schedule.xlsx
+++ b/docs/gantt_schedule.xlsx
@@ -507,11 +507,11 @@
   <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="5" customWidth="1" min="6" max="6"/>
     <col width="5" customWidth="1" min="7" max="7"/>
     <col width="5" customWidth="1" min="8" max="8"/>
@@ -822,7 +822,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Python 프로토타입</t>
+          <t>프로토타입 개발 방법론</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">

</xml_diff>